<commit_message>
Add June 21st match
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC5071DE-0C10-8244-8D2A-B1BC3783F96C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE699108-FD49-8245-A151-7834DA8370E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="1980" yWindow="9340" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="70">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -282,6 +282,42 @@
   </si>
   <si>
     <t>Netherlands</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jeremy Doku</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>repiratory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>thigh injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Giorgian De Arrascaeta</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>calf muscle injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Iran</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Roozbeh Cheshmi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Victor Munoz</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -669,11 +705,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="2" max="2" width="21.5" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
     <col min="4" max="4" width="31.1640625" customWidth="1"/>
     <col min="5" max="5" width="12.5" customWidth="1"/>
@@ -1139,6 +1175,126 @@
         <v>46194</v>
       </c>
     </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24">
+        <v>75</v>
+      </c>
+      <c r="D24" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24">
+        <v>-0.15</v>
+      </c>
+      <c r="F24" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25">
+        <v>28</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25">
+        <v>-0.05</v>
+      </c>
+      <c r="F25" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26">
+        <v>14</v>
+      </c>
+      <c r="D26" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26">
+        <v>-0.05</v>
+      </c>
+      <c r="F26" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27">
+        <v>-0.2</v>
+      </c>
+      <c r="F27" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28">
+        <v>0.45</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28">
+        <v>-0.1</v>
+      </c>
+      <c r="F28" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29">
+        <v>30</v>
+      </c>
+      <c r="D29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>-0.1</v>
+      </c>
+      <c r="F29" s="1">
+        <v>46194</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: fix home advantage issue
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE699108-FD49-8245-A151-7834DA8370E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5717F54F-68EA-1A4B-8F90-9B24AAC6E995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1980" yWindow="9340" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="200" yWindow="9620" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="101">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -318,6 +318,130 @@
   </si>
   <si>
     <t>Victor Munoz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gonzalo Montiel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mohamed Amoura</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>undisclosed injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Iraq</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Shammari</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tomas Araujo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Panama</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Adakberto Carrasquilla</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>groin injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ismael Kone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tibia and fibula fracture</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tarik Muharemovic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Qatar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Homam Ahmed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assim Madibo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Raphinha</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>grade-two hamstring injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Teboho Mokoena</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Czechia</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>David Jurasek</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Germany</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nico Schlotterbeck</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nathaniel Brown</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ankle ligament injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>minor muscular knock</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Australia</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacob Italiano</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adductor injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mathew Leckie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hamstring strain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Miguel Almiron</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -705,7 +829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -769,7 +893,7 @@
         <v>10</v>
       </c>
       <c r="E3">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="F3" s="1">
         <v>46185</v>
@@ -809,7 +933,7 @@
         <v>16</v>
       </c>
       <c r="E5">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F5" s="1">
         <v>46186</v>
@@ -849,7 +973,7 @@
         <v>22</v>
       </c>
       <c r="E7">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F7" s="1">
         <v>46187</v>
@@ -869,7 +993,7 @@
         <v>25</v>
       </c>
       <c r="E8">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F8" s="1">
         <v>46188</v>
@@ -889,7 +1013,7 @@
         <v>28</v>
       </c>
       <c r="E9">
-        <v>-0.25</v>
+        <v>-0.2</v>
       </c>
       <c r="F9" s="1">
         <v>46188</v>
@@ -929,7 +1053,7 @@
         <v>35</v>
       </c>
       <c r="E11">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F11" s="1">
         <v>46189</v>
@@ -969,7 +1093,7 @@
         <v>41</v>
       </c>
       <c r="E13">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="F13" s="1">
         <v>46190</v>
@@ -989,7 +1113,7 @@
         <v>44</v>
       </c>
       <c r="E14">
-        <v>-0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="F14" s="1">
         <v>46190</v>
@@ -1069,7 +1193,7 @@
         <v>47</v>
       </c>
       <c r="E18">
-        <v>-0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="F18" s="1">
         <v>46191</v>
@@ -1089,7 +1213,7 @@
         <v>16</v>
       </c>
       <c r="E19">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F19" s="1">
         <v>46192</v>
@@ -1129,7 +1253,7 @@
         <v>22</v>
       </c>
       <c r="E21">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F21" s="1">
         <v>46193</v>
@@ -1149,7 +1273,7 @@
         <v>56</v>
       </c>
       <c r="E22">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F22" s="1">
         <v>46193</v>
@@ -1269,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E28">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F28" s="1">
         <v>46194</v>
@@ -1289,10 +1413,410 @@
         <v>31</v>
       </c>
       <c r="E29">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F29" s="1">
         <v>46194</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30">
+        <v>-0.05</v>
+      </c>
+      <c r="F30" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31">
+        <v>22</v>
+      </c>
+      <c r="D31" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31">
+        <v>-0.05</v>
+      </c>
+      <c r="F31" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32">
+        <v>0.6</v>
+      </c>
+      <c r="D32" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32">
+        <v>-0.05</v>
+      </c>
+      <c r="F32" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33">
+        <v>30</v>
+      </c>
+      <c r="D33" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33">
+        <v>-0.05</v>
+      </c>
+      <c r="F33" s="1">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34" t="s">
+        <v>78</v>
+      </c>
+      <c r="E34">
+        <v>-0.2</v>
+      </c>
+      <c r="F34" s="1">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35">
+        <v>25</v>
+      </c>
+      <c r="D35" t="s">
+        <v>80</v>
+      </c>
+      <c r="E35">
+        <v>-0.2</v>
+      </c>
+      <c r="F35" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36">
+        <v>-0.05</v>
+      </c>
+      <c r="F36" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37">
+        <v>25</v>
+      </c>
+      <c r="D37" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37">
+        <v>-0.05</v>
+      </c>
+      <c r="F37" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>82</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38">
+        <v>0.45</v>
+      </c>
+      <c r="D38" t="s">
+        <v>47</v>
+      </c>
+      <c r="E38">
+        <v>-0.1</v>
+      </c>
+      <c r="F38" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39">
+        <v>0.3</v>
+      </c>
+      <c r="D39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39">
+        <v>-0.2</v>
+      </c>
+      <c r="F39" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" t="s">
+        <v>85</v>
+      </c>
+      <c r="C40">
+        <v>80</v>
+      </c>
+      <c r="D40" t="s">
+        <v>86</v>
+      </c>
+      <c r="E40">
+        <v>-0.05</v>
+      </c>
+      <c r="F40" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41">
+        <v>2.4</v>
+      </c>
+      <c r="D41" t="s">
+        <v>47</v>
+      </c>
+      <c r="E41">
+        <v>-0.05</v>
+      </c>
+      <c r="F41" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" t="s">
+        <v>46</v>
+      </c>
+      <c r="C42">
+        <v>0.25</v>
+      </c>
+      <c r="D42" t="s">
+        <v>47</v>
+      </c>
+      <c r="E42">
+        <v>-0.05</v>
+      </c>
+      <c r="F42" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>31</v>
+      </c>
+      <c r="E43">
+        <v>-0.05</v>
+      </c>
+      <c r="F43" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44">
+        <v>55</v>
+      </c>
+      <c r="D44" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44">
+        <v>-0.05</v>
+      </c>
+      <c r="F44" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45">
+        <v>40</v>
+      </c>
+      <c r="D45" t="s">
+        <v>94</v>
+      </c>
+      <c r="E45">
+        <v>-0.05</v>
+      </c>
+      <c r="F45" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>57</v>
+      </c>
+      <c r="B46" t="s">
+        <v>58</v>
+      </c>
+      <c r="C46">
+        <v>20</v>
+      </c>
+      <c r="D46" t="s">
+        <v>59</v>
+      </c>
+      <c r="E46">
+        <v>-0.05</v>
+      </c>
+      <c r="F46" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>95</v>
+      </c>
+      <c r="B47" t="s">
+        <v>96</v>
+      </c>
+      <c r="C47">
+        <v>0.6</v>
+      </c>
+      <c r="D47" t="s">
+        <v>97</v>
+      </c>
+      <c r="E47">
+        <v>-0.05</v>
+      </c>
+      <c r="F47" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48" t="s">
+        <v>98</v>
+      </c>
+      <c r="C48">
+        <v>0.3</v>
+      </c>
+      <c r="D48" t="s">
+        <v>99</v>
+      </c>
+      <c r="E48">
+        <v>-0.1</v>
+      </c>
+      <c r="F48" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49">
+        <v>7</v>
+      </c>
+      <c r="D49" t="s">
+        <v>47</v>
+      </c>
+      <c r="E49">
+        <v>-0.15</v>
+      </c>
+      <c r="F49" s="1">
+        <v>46198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update result until end of group stage
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5717F54F-68EA-1A4B-8F90-9B24AAC6E995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB098A20-641A-E240-926B-EC5D866829D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="200" yWindow="9620" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -442,6 +442,90 @@
   </si>
   <si>
     <t>Miguel Almiron</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Norway</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Julian Ryerson</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>France</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>William Saliba</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>back issue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Senegal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Edouard Mendy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cape Verde</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sidny Lopes Cabral</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>muscle strain injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Egypt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hamdi Fathi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hossam Abdelmaguid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>head injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nathan Ngoy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lawrence Ati-Zigi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>England</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reece James</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>minor hamstring injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cristian Romero</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>knee injury</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -829,7 +913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -1819,6 +1903,326 @@
         <v>46198</v>
       </c>
     </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50">
+        <v>100</v>
+      </c>
+      <c r="D50" t="s">
+        <v>105</v>
+      </c>
+      <c r="E50">
+        <v>-0.1</v>
+      </c>
+      <c r="F50" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B51" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51">
+        <v>25</v>
+      </c>
+      <c r="D51" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51">
+        <v>-0.05</v>
+      </c>
+      <c r="F51" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" t="s">
+        <v>106</v>
+      </c>
+      <c r="B52" t="s">
+        <v>107</v>
+      </c>
+      <c r="C52">
+        <v>4</v>
+      </c>
+      <c r="D52" t="s">
+        <v>59</v>
+      </c>
+      <c r="E52">
+        <v>-0.05</v>
+      </c>
+      <c r="F52" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+      <c r="D53" t="s">
+        <v>47</v>
+      </c>
+      <c r="E53">
+        <v>-0.05</v>
+      </c>
+      <c r="F53" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>26</v>
+      </c>
+      <c r="B54" t="s">
+        <v>27</v>
+      </c>
+      <c r="C54">
+        <v>20</v>
+      </c>
+      <c r="D54" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54">
+        <v>-0.2</v>
+      </c>
+      <c r="F54" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>26</v>
+      </c>
+      <c r="B55" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55">
+        <v>14</v>
+      </c>
+      <c r="D55" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55">
+        <v>-0.05</v>
+      </c>
+      <c r="F55" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" t="s">
+        <v>68</v>
+      </c>
+      <c r="B56" t="s">
+        <v>69</v>
+      </c>
+      <c r="C56">
+        <v>30</v>
+      </c>
+      <c r="D56" t="s">
+        <v>110</v>
+      </c>
+      <c r="E56">
+        <v>-0.05</v>
+      </c>
+      <c r="F56" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>111</v>
+      </c>
+      <c r="B57" t="s">
+        <v>112</v>
+      </c>
+      <c r="C57">
+        <v>1.8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>31</v>
+      </c>
+      <c r="E57">
+        <v>-0.05</v>
+      </c>
+      <c r="F57" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>111</v>
+      </c>
+      <c r="B58" t="s">
+        <v>113</v>
+      </c>
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58" t="s">
+        <v>114</v>
+      </c>
+      <c r="E58">
+        <v>-0.05</v>
+      </c>
+      <c r="F58" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>23</v>
+      </c>
+      <c r="B59" t="s">
+        <v>115</v>
+      </c>
+      <c r="C59">
+        <v>25</v>
+      </c>
+      <c r="D59" t="s">
+        <v>47</v>
+      </c>
+      <c r="E59">
+        <v>-0.05</v>
+      </c>
+      <c r="F59" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>42</v>
+      </c>
+      <c r="B60" t="s">
+        <v>116</v>
+      </c>
+      <c r="C60">
+        <v>1.5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E60">
+        <v>-0.05</v>
+      </c>
+      <c r="F60" s="1">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" t="s">
+        <v>118</v>
+      </c>
+      <c r="C61">
+        <v>60</v>
+      </c>
+      <c r="D61" t="s">
+        <v>119</v>
+      </c>
+      <c r="E61">
+        <v>-0.05</v>
+      </c>
+      <c r="F61" s="1">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>76</v>
+      </c>
+      <c r="B62" t="s">
+        <v>77</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+      <c r="D62" t="s">
+        <v>31</v>
+      </c>
+      <c r="E62">
+        <v>-0.2</v>
+      </c>
+      <c r="F62" s="1">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>33</v>
+      </c>
+      <c r="B63" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63">
+        <v>45</v>
+      </c>
+      <c r="D63" t="s">
+        <v>121</v>
+      </c>
+      <c r="E63">
+        <v>-0.05</v>
+      </c>
+      <c r="F63" s="1">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>8</v>
+      </c>
+      <c r="B64" t="s">
+        <v>79</v>
+      </c>
+      <c r="C64">
+        <v>25</v>
+      </c>
+      <c r="D64" t="s">
+        <v>80</v>
+      </c>
+      <c r="E64">
+        <v>-0.1</v>
+      </c>
+      <c r="F64" s="1">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" t="s">
+        <v>45</v>
+      </c>
+      <c r="B65" t="s">
+        <v>46</v>
+      </c>
+      <c r="C65">
+        <v>0.25</v>
+      </c>
+      <c r="D65" t="s">
+        <v>47</v>
+      </c>
+      <c r="E65">
+        <v>-0.05</v>
+      </c>
+      <c r="F65" s="1">
+        <v>46201</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add exact score prediction on match details page
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB098A20-641A-E240-926B-EC5D866829D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5990A68-2211-054B-92C3-AEC04BCC44DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="124">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -526,6 +526,14 @@
   </si>
   <si>
     <t>knee injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>left ankle tear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Diego Gomez</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -913,7 +921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -2223,6 +2231,86 @@
         <v>46201</v>
       </c>
     </row>
+    <row r="66" spans="1:6">
+      <c r="A66" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66" t="s">
+        <v>85</v>
+      </c>
+      <c r="C66">
+        <v>80</v>
+      </c>
+      <c r="D66" t="s">
+        <v>10</v>
+      </c>
+      <c r="E66">
+        <v>-0.05</v>
+      </c>
+      <c r="F66" s="1">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" t="s">
+        <v>57</v>
+      </c>
+      <c r="B67" t="s">
+        <v>58</v>
+      </c>
+      <c r="C67">
+        <v>20</v>
+      </c>
+      <c r="D67" t="s">
+        <v>59</v>
+      </c>
+      <c r="E67">
+        <v>-0.05</v>
+      </c>
+      <c r="F67" s="1">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>90</v>
+      </c>
+      <c r="B68" t="s">
+        <v>91</v>
+      </c>
+      <c r="C68">
+        <v>55</v>
+      </c>
+      <c r="D68" t="s">
+        <v>122</v>
+      </c>
+      <c r="E68">
+        <v>-0.05</v>
+      </c>
+      <c r="F68" s="1">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" t="s">
+        <v>52</v>
+      </c>
+      <c r="B69" t="s">
+        <v>123</v>
+      </c>
+      <c r="C69">
+        <v>25</v>
+      </c>
+      <c r="D69" t="s">
+        <v>47</v>
+      </c>
+      <c r="E69">
+        <v>-0.2</v>
+      </c>
+      <c r="F69" s="1">
+        <v>46202</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: UI improvement and extend google sheet columns
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5990A68-2211-054B-92C3-AEC04BCC44DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E4C5B4-9173-4D49-BB06-0AA8268BD0A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="1060" yWindow="8240" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="142">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -534,6 +534,78 @@
   </si>
   <si>
     <t>Diego Gomez</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wilfried Singo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sweden</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Isak Hien</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Marcus Thuram</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jarell Quansah</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>twisted ankle</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nico Williams</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yeremy Pino</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ruptured collarbone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Austria</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Phillipp Mwene</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ahmed Fattouh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hamstring tear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mohanad Lasheen</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Telmo Arcanjo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kojo Oppong Peprah</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>training injury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Aurelien Tchouameni</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -921,7 +993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -1165,7 +1237,7 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="F12" s="1">
         <v>46189</v>
@@ -1345,7 +1417,7 @@
         <v>22</v>
       </c>
       <c r="E21">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="F21" s="1">
         <v>46193</v>
@@ -1465,7 +1537,7 @@
         <v>28</v>
       </c>
       <c r="E27">
-        <v>-0.2</v>
+        <v>-0.15</v>
       </c>
       <c r="F27" s="1">
         <v>46194</v>
@@ -1625,7 +1697,7 @@
         <v>80</v>
       </c>
       <c r="E35">
-        <v>-0.2</v>
+        <v>-0.15</v>
       </c>
       <c r="F35" s="1">
         <v>46197</v>
@@ -1685,7 +1757,7 @@
         <v>47</v>
       </c>
       <c r="E38">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F38" s="1">
         <v>46197</v>
@@ -1925,7 +1997,7 @@
         <v>105</v>
       </c>
       <c r="E50">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="F50" s="1">
         <v>46199</v>
@@ -1945,7 +2017,7 @@
         <v>63</v>
       </c>
       <c r="E51">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="F51" s="1">
         <v>46199</v>
@@ -2309,6 +2381,406 @@
       </c>
       <c r="F69" s="1">
         <v>46202</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" t="s">
+        <v>21</v>
+      </c>
+      <c r="B70" t="s">
+        <v>124</v>
+      </c>
+      <c r="C70">
+        <v>23</v>
+      </c>
+      <c r="D70" t="s">
+        <v>10</v>
+      </c>
+      <c r="E70">
+        <v>-0.05</v>
+      </c>
+      <c r="F70" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" t="s">
+        <v>101</v>
+      </c>
+      <c r="B71" t="s">
+        <v>102</v>
+      </c>
+      <c r="C71">
+        <v>25</v>
+      </c>
+      <c r="D71" t="s">
+        <v>63</v>
+      </c>
+      <c r="E71">
+        <v>-0.05</v>
+      </c>
+      <c r="F71" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" t="s">
+        <v>125</v>
+      </c>
+      <c r="B72" t="s">
+        <v>126</v>
+      </c>
+      <c r="C72">
+        <v>22</v>
+      </c>
+      <c r="D72" t="s">
+        <v>10</v>
+      </c>
+      <c r="E72">
+        <v>-0.2</v>
+      </c>
+      <c r="F72" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" t="s">
+        <v>103</v>
+      </c>
+      <c r="B73" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73">
+        <v>50</v>
+      </c>
+      <c r="D73" t="s">
+        <v>19</v>
+      </c>
+      <c r="E73">
+        <v>-0.05</v>
+      </c>
+      <c r="F73" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" t="s">
+        <v>117</v>
+      </c>
+      <c r="B74" t="s">
+        <v>118</v>
+      </c>
+      <c r="C74">
+        <v>60</v>
+      </c>
+      <c r="D74" t="s">
+        <v>10</v>
+      </c>
+      <c r="E74">
+        <v>-0.03</v>
+      </c>
+      <c r="F74" s="1">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" t="s">
+        <v>117</v>
+      </c>
+      <c r="B75" t="s">
+        <v>128</v>
+      </c>
+      <c r="C75">
+        <v>45</v>
+      </c>
+      <c r="D75" t="s">
+        <v>129</v>
+      </c>
+      <c r="E75">
+        <v>-0.02</v>
+      </c>
+      <c r="F75" s="1">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" t="s">
+        <v>106</v>
+      </c>
+      <c r="B76" t="s">
+        <v>107</v>
+      </c>
+      <c r="C76">
+        <v>4</v>
+      </c>
+      <c r="D76" t="s">
+        <v>121</v>
+      </c>
+      <c r="E76">
+        <v>-0.1</v>
+      </c>
+      <c r="F76" s="1">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" t="s">
+        <v>68</v>
+      </c>
+      <c r="B77" t="s">
+        <v>130</v>
+      </c>
+      <c r="C77">
+        <v>40</v>
+      </c>
+      <c r="D77" t="s">
+        <v>31</v>
+      </c>
+      <c r="E77">
+        <v>-0.05</v>
+      </c>
+      <c r="F77" s="1">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" t="s">
+        <v>68</v>
+      </c>
+      <c r="B78" t="s">
+        <v>131</v>
+      </c>
+      <c r="C78">
+        <v>30</v>
+      </c>
+      <c r="D78" t="s">
+        <v>132</v>
+      </c>
+      <c r="E78">
+        <v>-0.05</v>
+      </c>
+      <c r="F78" s="1">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" t="s">
+        <v>133</v>
+      </c>
+      <c r="B79" t="s">
+        <v>134</v>
+      </c>
+      <c r="C79">
+        <v>1.5</v>
+      </c>
+      <c r="D79" t="s">
+        <v>63</v>
+      </c>
+      <c r="E79">
+        <v>-0.2</v>
+      </c>
+      <c r="F79" s="1">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" t="s">
+        <v>36</v>
+      </c>
+      <c r="B80" t="s">
+        <v>71</v>
+      </c>
+      <c r="C80">
+        <v>20</v>
+      </c>
+      <c r="D80" t="s">
+        <v>72</v>
+      </c>
+      <c r="E80">
+        <v>-0.1</v>
+      </c>
+      <c r="F80" s="1">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" t="s">
+        <v>111</v>
+      </c>
+      <c r="B81" t="s">
+        <v>135</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81" t="s">
+        <v>136</v>
+      </c>
+      <c r="E81">
+        <v>-0.05</v>
+      </c>
+      <c r="F81" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82" t="s">
+        <v>137</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82" t="s">
+        <v>47</v>
+      </c>
+      <c r="E82">
+        <v>-0.05</v>
+      </c>
+      <c r="F82" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" t="s">
+        <v>95</v>
+      </c>
+      <c r="B83" t="s">
+        <v>98</v>
+      </c>
+      <c r="C83">
+        <v>0.3</v>
+      </c>
+      <c r="D83" t="s">
+        <v>10</v>
+      </c>
+      <c r="E83">
+        <v>-0.1</v>
+      </c>
+      <c r="F83" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" t="s">
+        <v>95</v>
+      </c>
+      <c r="B84" t="s">
+        <v>96</v>
+      </c>
+      <c r="C84">
+        <v>0.6</v>
+      </c>
+      <c r="D84" t="s">
+        <v>78</v>
+      </c>
+      <c r="E84">
+        <v>-0.05</v>
+      </c>
+      <c r="F84" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" t="s">
+        <v>108</v>
+      </c>
+      <c r="B85" t="s">
+        <v>138</v>
+      </c>
+      <c r="C85">
+        <v>3</v>
+      </c>
+      <c r="D85" t="s">
+        <v>10</v>
+      </c>
+      <c r="E85">
+        <v>-0.1</v>
+      </c>
+      <c r="F85" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" t="s">
+        <v>42</v>
+      </c>
+      <c r="B86" t="s">
+        <v>139</v>
+      </c>
+      <c r="C86">
+        <v>10</v>
+      </c>
+      <c r="D86" t="s">
+        <v>140</v>
+      </c>
+      <c r="E86">
+        <v>-0.05</v>
+      </c>
+      <c r="F86" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" t="s">
+        <v>8</v>
+      </c>
+      <c r="B87" t="s">
+        <v>79</v>
+      </c>
+      <c r="C87">
+        <v>25</v>
+      </c>
+      <c r="D87" t="s">
+        <v>80</v>
+      </c>
+      <c r="E87">
+        <v>-0.15</v>
+      </c>
+      <c r="F87" s="1">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" t="s">
+        <v>103</v>
+      </c>
+      <c r="B88" t="s">
+        <v>141</v>
+      </c>
+      <c r="C88">
+        <v>70</v>
+      </c>
+      <c r="D88" t="s">
+        <v>63</v>
+      </c>
+      <c r="E88">
+        <v>-0.03</v>
+      </c>
+      <c r="F88" s="1">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" t="s">
+        <v>103</v>
+      </c>
+      <c r="B89" t="s">
+        <v>127</v>
+      </c>
+      <c r="C89">
+        <v>50</v>
+      </c>
+      <c r="D89" t="s">
+        <v>35</v>
+      </c>
+      <c r="E89">
+        <v>-0.02</v>
+      </c>
+      <c r="F89" s="1">
+        <v>46207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add value_lab section
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E4C5B4-9173-4D49-BB06-0AA8268BD0A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8841E098-9E83-4945-9B2C-449B5339D31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="8240" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="0" yWindow="2700" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="149">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -606,6 +606,34 @@
   </si>
   <si>
     <t>Aurelien Tchouameni</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lucas Paqueta</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Colombia</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jhon Cordoba</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Switzerland</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Luca Jaquez</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Morocco</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ismael Saibari</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -993,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -2783,6 +2811,106 @@
         <v>46207</v>
       </c>
     </row>
+    <row r="90" spans="1:6">
+      <c r="A90" t="s">
+        <v>14</v>
+      </c>
+      <c r="B90" t="s">
+        <v>142</v>
+      </c>
+      <c r="C90">
+        <v>32</v>
+      </c>
+      <c r="D90" t="s">
+        <v>10</v>
+      </c>
+      <c r="E90">
+        <v>-0.05</v>
+      </c>
+      <c r="F90" s="1">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" t="s">
+        <v>111</v>
+      </c>
+      <c r="B91" t="s">
+        <v>135</v>
+      </c>
+      <c r="C91">
+        <v>1</v>
+      </c>
+      <c r="D91" t="s">
+        <v>136</v>
+      </c>
+      <c r="E91">
+        <v>-0.1</v>
+      </c>
+      <c r="F91" s="1">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" t="s">
+        <v>143</v>
+      </c>
+      <c r="B92" t="s">
+        <v>144</v>
+      </c>
+      <c r="C92">
+        <v>10</v>
+      </c>
+      <c r="D92" t="s">
+        <v>99</v>
+      </c>
+      <c r="E92">
+        <v>-0.05</v>
+      </c>
+      <c r="F92" s="1">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" t="s">
+        <v>145</v>
+      </c>
+      <c r="B93" t="s">
+        <v>146</v>
+      </c>
+      <c r="C93">
+        <v>10</v>
+      </c>
+      <c r="D93" t="s">
+        <v>72</v>
+      </c>
+      <c r="E93">
+        <v>-0.05</v>
+      </c>
+      <c r="F93" s="1">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" t="s">
+        <v>147</v>
+      </c>
+      <c r="B94" t="s">
+        <v>148</v>
+      </c>
+      <c r="C94">
+        <v>40</v>
+      </c>
+      <c r="D94" t="s">
+        <v>10</v>
+      </c>
+      <c r="E94">
+        <v>-0.1</v>
+      </c>
+      <c r="F94" s="1">
+        <v>46212</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update match until July 11th
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8841E098-9E83-4945-9B2C-449B5339D31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82B338D-E4A0-6045-8CF0-C771F8AE8C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2700" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="155">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -634,6 +634,30 @@
   </si>
   <si>
     <t>Ismael Saibari</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Amadou Onana</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ACL right knee</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>medical fitness dispute</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jordan Henderson</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>broken arm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Johan Manzambi</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1021,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -2911,6 +2935,126 @@
         <v>46212</v>
       </c>
     </row>
+    <row r="95" spans="1:6">
+      <c r="A95" t="s">
+        <v>68</v>
+      </c>
+      <c r="B95" t="s">
+        <v>131</v>
+      </c>
+      <c r="C95">
+        <v>30</v>
+      </c>
+      <c r="D95" t="s">
+        <v>132</v>
+      </c>
+      <c r="E95">
+        <v>-0.05</v>
+      </c>
+      <c r="F95" s="1">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" t="s">
+        <v>23</v>
+      </c>
+      <c r="B96" t="s">
+        <v>149</v>
+      </c>
+      <c r="C96">
+        <v>45</v>
+      </c>
+      <c r="D96" t="s">
+        <v>150</v>
+      </c>
+      <c r="E96">
+        <v>-0.15</v>
+      </c>
+      <c r="F96" s="1">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" t="s">
+        <v>23</v>
+      </c>
+      <c r="B97" t="s">
+        <v>24</v>
+      </c>
+      <c r="C97">
+        <v>28</v>
+      </c>
+      <c r="D97" t="s">
+        <v>151</v>
+      </c>
+      <c r="E97">
+        <v>-0.05</v>
+      </c>
+      <c r="F97" s="1">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" t="s">
+        <v>117</v>
+      </c>
+      <c r="B98" t="s">
+        <v>152</v>
+      </c>
+      <c r="C98">
+        <v>1.2</v>
+      </c>
+      <c r="D98" t="s">
+        <v>153</v>
+      </c>
+      <c r="E98">
+        <v>-0.02</v>
+      </c>
+      <c r="F98" s="1">
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" t="s">
+        <v>117</v>
+      </c>
+      <c r="B99" t="s">
+        <v>128</v>
+      </c>
+      <c r="C99">
+        <v>45</v>
+      </c>
+      <c r="D99" t="s">
+        <v>47</v>
+      </c>
+      <c r="E99">
+        <v>-0.03</v>
+      </c>
+      <c r="F99" s="1">
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" t="s">
+        <v>145</v>
+      </c>
+      <c r="B100" t="s">
+        <v>154</v>
+      </c>
+      <c r="C100">
+        <v>50</v>
+      </c>
+      <c r="D100" t="s">
+        <v>121</v>
+      </c>
+      <c r="E100">
+        <v>-0.2</v>
+      </c>
+      <c r="F100" s="1">
+        <v>46214</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update claude settings
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82B338D-E4A0-6045-8CF0-C771F8AE8C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD518B5D-F257-C143-A619-610D5F020E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="155">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1045,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -3055,6 +3055,46 @@
         <v>46214</v>
       </c>
     </row>
+    <row r="101" spans="1:6">
+      <c r="A101" t="s">
+        <v>117</v>
+      </c>
+      <c r="B101" t="s">
+        <v>152</v>
+      </c>
+      <c r="C101">
+        <v>1.2</v>
+      </c>
+      <c r="D101" t="s">
+        <v>153</v>
+      </c>
+      <c r="E101">
+        <v>-0.02</v>
+      </c>
+      <c r="F101" s="1">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" t="s">
+        <v>117</v>
+      </c>
+      <c r="B102" t="s">
+        <v>128</v>
+      </c>
+      <c r="C102">
+        <v>45</v>
+      </c>
+      <c r="D102" t="s">
+        <v>47</v>
+      </c>
+      <c r="E102">
+        <v>-0.03</v>
+      </c>
+      <c r="F102" s="1">
+        <v>46218</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update world cup until end
</commit_message>
<xml_diff>
--- a/data/Injury_report.xlsx
+++ b/data/Injury_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuyuchuan/Desktop/Soccer/World_Cup/decision_copilot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD518B5D-F257-C143-A619-610D5F020E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07835ADD-4F6F-7B4C-A759-84821FBC462E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="28800" windowHeight="16240" xr2:uid="{5174A3A6-D970-F447-9BEE-F4196D91B1B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="155">
   <si>
     <t>team</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1045,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BBFD96D-7402-BC4B-B112-DE0E5BDC66F2}">
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -3095,6 +3095,66 @@
         <v>46218</v>
       </c>
     </row>
+    <row r="103" spans="1:6">
+      <c r="A103" t="s">
+        <v>103</v>
+      </c>
+      <c r="B103" t="s">
+        <v>104</v>
+      </c>
+      <c r="C103">
+        <v>100</v>
+      </c>
+      <c r="D103" t="s">
+        <v>105</v>
+      </c>
+      <c r="E103">
+        <v>-0.05</v>
+      </c>
+      <c r="F103" s="1">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" t="s">
+        <v>117</v>
+      </c>
+      <c r="B104" t="s">
+        <v>152</v>
+      </c>
+      <c r="C104">
+        <v>1.2</v>
+      </c>
+      <c r="D104" t="s">
+        <v>153</v>
+      </c>
+      <c r="E104">
+        <v>-0.05</v>
+      </c>
+      <c r="F104" s="1">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" t="s">
+        <v>117</v>
+      </c>
+      <c r="B105" t="s">
+        <v>118</v>
+      </c>
+      <c r="C105">
+        <v>60</v>
+      </c>
+      <c r="D105" t="s">
+        <v>54</v>
+      </c>
+      <c r="E105">
+        <v>-0.1</v>
+      </c>
+      <c r="F105" s="1">
+        <v>46221</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>